<commit_message>
Update spreadsheet files across finance sections
</commit_message>
<xml_diff>
--- a/sheets/investing/dca-vs-lump-sum/dca-vs-lump-sum.xlsx
+++ b/sheets/investing/dca-vs-lump-sum/dca-vs-lump-sum.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\000_drive_drive\600_PROJECTS\modelstack\sheets\investing\dca-vs-lump-sum\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\My Drive\000_drive_drive\600_PROJECTS\modelstack\sheets\investing\dca-vs-lump-sum\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA30B7B9-BDD2-4113-BD9F-9C0AA54DFD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54635C1-B00A-497C-972E-FE5D84EB8CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Price History" sheetId="1" r:id="rId1"/>
@@ -131,10 +131,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,8 +161,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF4472C4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -186,7 +200,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F2E8"/>
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -217,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -234,53 +255,46 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -348,26 +362,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1">
-                  <a:lumMod val="50000"/>
-                  <a:lumOff val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -860,26 +854,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1052,26 +1026,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="20" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1">
-                  <a:lumMod val="50000"/>
-                  <a:lumOff val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -1564,26 +1518,6 @@
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
         </c:title>
         <c:numFmt formatCode="&quot;$&quot;#,##0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
@@ -1756,26 +1690,6 @@
         </a:ln>
         <a:effectLst/>
       </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="150" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="50000"/>
-                  <a:lumOff val="50000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
@@ -2336,6 +2250,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="2035262832"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
         <c:baseTimeUnit val="months"/>
@@ -2424,1721 +2339,6 @@
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="230">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" b="0" kern="1200" spc="20" baseline="0"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="1"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="1"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="22225" cap="rnd" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-            <a:alpha val="33000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:gradFill>
-        <a:gsLst>
-          <a:gs pos="100000">
-            <a:schemeClr val="lt1">
-              <a:lumMod val="95000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="0">
-            <a:schemeClr val="lt1"/>
-          </a:gs>
-        </a:gsLst>
-        <a:lin ang="5400000" scaled="0"/>
-      </a:gradFill>
-    </cs:spPr>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" kern="1200" cap="none" spc="20" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" spc="20" baseline="0"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="230">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" b="0" kern="1200" spc="20" baseline="0"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="1"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="2">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="1"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:shade val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="22225" cap="rnd" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-            <a:alpha val="33000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:gradFill>
-        <a:gsLst>
-          <a:gs pos="100000">
-            <a:schemeClr val="lt1">
-              <a:lumMod val="95000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="0">
-            <a:schemeClr val="lt1"/>
-          </a:gs>
-        </a:gsLst>
-        <a:lin ang="5400000" scaled="0"/>
-      </a:gradFill>
-    </cs:spPr>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" kern="1200" cap="none" spc="20" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" spc="20" baseline="0"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="203">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="narHorz">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="20000"/>
-            <a:lumOff val="80000"/>
-          </a:schemeClr>
-        </a:bgClr>
-      </a:pattFill>
-      <a:effectLst>
-        <a:innerShdw blurRad="114300">
-          <a:schemeClr val="phClr"/>
-        </a:innerShdw>
-      </a:effectLst>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="50000"/>
-        <a:lumOff val="50000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4528,7 +2728,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
@@ -4537,7 +2737,7 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20">
+      <c r="B1" s="14">
         <v>500</v>
       </c>
       <c r="C1" s="1"/>
@@ -4550,14 +2750,14 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="15">
         <v>45322</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="18">
         <f>COUNTA(A7:A30)</f>
         <v>24</v>
       </c>
@@ -4566,33 +2766,33 @@
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="21">
+      <c r="B3" s="15">
         <v>46022</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="19">
         <f>AVERAGE(B7:B30)</f>
         <v>112.04166666666667</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="14"/>
+      <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="19">
         <f>MAX(B7:B30)-MIN(B7:B30)</f>
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="14"/>
+      <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -4601,7 +2801,7 @@
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="1"/>
@@ -4612,7 +2812,7 @@
       <c r="A7" s="4">
         <v>45322</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="16">
         <v>102</v>
       </c>
       <c r="C7" s="1"/>
@@ -4623,7 +2823,7 @@
       <c r="A8" s="4">
         <v>45351</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="16">
         <v>97</v>
       </c>
       <c r="C8" s="1"/>
@@ -4634,7 +2834,7 @@
       <c r="A9" s="4">
         <v>45382</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="16">
         <v>94</v>
       </c>
       <c r="C9" s="1"/>
@@ -4645,7 +2845,7 @@
       <c r="A10" s="4">
         <v>45412</v>
       </c>
-      <c r="B10" s="22">
+      <c r="B10" s="16">
         <v>99</v>
       </c>
       <c r="C10" s="1"/>
@@ -4656,7 +2856,7 @@
       <c r="A11" s="4">
         <v>45443</v>
       </c>
-      <c r="B11" s="22">
+      <c r="B11" s="16">
         <v>104</v>
       </c>
       <c r="C11" s="1"/>
@@ -4667,7 +2867,7 @@
       <c r="A12" s="4">
         <v>45473</v>
       </c>
-      <c r="B12" s="22">
+      <c r="B12" s="16">
         <v>108</v>
       </c>
       <c r="C12" s="1"/>
@@ -4678,7 +2878,7 @@
       <c r="A13" s="4">
         <v>45504</v>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="16">
         <v>111</v>
       </c>
       <c r="C13" s="1"/>
@@ -4689,7 +2889,7 @@
       <c r="A14" s="4">
         <v>45535</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="16">
         <v>109</v>
       </c>
       <c r="C14" s="1"/>
@@ -4700,7 +2900,7 @@
       <c r="A15" s="4">
         <v>45565</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="16">
         <v>105</v>
       </c>
       <c r="C15" s="1"/>
@@ -4711,7 +2911,7 @@
       <c r="A16" s="4">
         <v>45596</v>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="16">
         <v>101</v>
       </c>
       <c r="C16" s="1"/>
@@ -4722,7 +2922,7 @@
       <c r="A17" s="4">
         <v>45626</v>
       </c>
-      <c r="B17" s="22">
+      <c r="B17" s="16">
         <v>98</v>
       </c>
       <c r="C17" s="1"/>
@@ -4733,7 +2933,7 @@
       <c r="A18" s="4">
         <v>45657</v>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="16">
         <v>103</v>
       </c>
       <c r="C18" s="1"/>
@@ -4744,7 +2944,7 @@
       <c r="A19" s="4">
         <v>45688</v>
       </c>
-      <c r="B19" s="22">
+      <c r="B19" s="16">
         <v>107</v>
       </c>
       <c r="C19" s="1"/>
@@ -4755,7 +2955,7 @@
       <c r="A20" s="4">
         <v>45716</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="16">
         <v>112</v>
       </c>
       <c r="C20" s="1"/>
@@ -4766,7 +2966,7 @@
       <c r="A21" s="4">
         <v>45747</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="16">
         <v>116</v>
       </c>
       <c r="C21" s="1"/>
@@ -4777,7 +2977,7 @@
       <c r="A22" s="4">
         <v>45777</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="16">
         <v>114</v>
       </c>
       <c r="C22" s="1"/>
@@ -4788,7 +2988,7 @@
       <c r="A23" s="4">
         <v>45808</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="16">
         <v>118</v>
       </c>
       <c r="C23" s="1"/>
@@ -4799,7 +2999,7 @@
       <c r="A24" s="4">
         <v>45838</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="16">
         <v>121</v>
       </c>
       <c r="C24" s="1"/>
@@ -4810,7 +3010,7 @@
       <c r="A25" s="4">
         <v>45869</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="16">
         <v>125</v>
       </c>
       <c r="C25" s="1"/>
@@ -4821,7 +3021,7 @@
       <c r="A26" s="4">
         <v>45900</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="16">
         <v>123</v>
       </c>
       <c r="C26" s="1"/>
@@ -4832,7 +3032,7 @@
       <c r="A27" s="4">
         <v>45930</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="16">
         <v>128</v>
       </c>
       <c r="C27" s="1"/>
@@ -4843,7 +3043,7 @@
       <c r="A28" s="4">
         <v>45961</v>
       </c>
-      <c r="B28" s="22">
+      <c r="B28" s="16">
         <v>131</v>
       </c>
       <c r="C28" s="1"/>
@@ -4854,7 +3054,7 @@
       <c r="A29" s="4">
         <v>45991</v>
       </c>
-      <c r="B29" s="22">
+      <c r="B29" s="16">
         <v>129</v>
       </c>
       <c r="C29" s="1"/>
@@ -4865,7 +3065,7 @@
       <c r="A30" s="4">
         <v>46022</v>
       </c>
-      <c r="B30" s="22">
+      <c r="B30" s="16">
         <v>134</v>
       </c>
       <c r="C30" s="1"/>
@@ -4883,21 +3083,15 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -4923,919 +3117,952 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="6">
         <f>'Price History'!A7</f>
         <v>45322</v>
       </c>
-      <c r="B2" s="19">
+      <c r="B2" s="7">
         <f>'Price History'!B7</f>
         <v>102</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="9">
         <f t="shared" ref="D2:D25" si="0">C2/B2</f>
         <v>4.9019607843137258</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="9">
         <f>D2</f>
         <v>4.9019607843137258</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="8">
         <f>C2</f>
         <v>500</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="7">
         <f t="shared" ref="G2:G25" si="1">IF(E2=0,0,F2/E2)</f>
         <v>101.99999999999999</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="8">
         <f t="shared" ref="H2:H25" si="2">E2*B2</f>
         <v>500.00000000000006</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="8">
         <f t="shared" ref="I2:I25" si="3">H2-F2</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="6">
         <f>'Price History'!A8</f>
         <v>45351</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="7">
         <f>'Price History'!B8</f>
         <v>97</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="9">
         <f t="shared" si="0"/>
         <v>5.1546391752577323</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="9">
         <f t="shared" ref="E3:E25" si="4">E2+D3</f>
         <v>10.056599959571457</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="8">
         <f t="shared" ref="F3:F25" si="5">F2+C3</f>
         <v>1000</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="7">
         <f t="shared" si="1"/>
         <v>99.437185929648237</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="8">
         <f t="shared" si="2"/>
         <v>975.49019607843138</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="8">
         <f t="shared" si="3"/>
         <v>-24.509803921568619</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="6">
         <f>'Price History'!A9</f>
         <v>45382</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="7">
         <f>'Price History'!B9</f>
         <v>94</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="9">
         <f t="shared" si="0"/>
         <v>5.3191489361702127</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="9">
         <f t="shared" si="4"/>
         <v>15.375748895741669</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="8">
         <f t="shared" si="5"/>
         <v>1500</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="7">
         <f t="shared" si="1"/>
         <v>97.556223776223788</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="8">
         <f t="shared" si="2"/>
         <v>1445.3203961997169</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="8">
         <f t="shared" si="3"/>
         <v>-54.679603800283076</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <f>'Price History'!A10</f>
         <v>45412</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="7">
         <f>'Price History'!B10</f>
         <v>99</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="9">
         <f t="shared" si="0"/>
         <v>5.0505050505050502</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="9">
         <f t="shared" si="4"/>
         <v>20.426253946246717</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="8">
         <f t="shared" si="5"/>
         <v>2000</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="7">
         <f t="shared" si="1"/>
         <v>97.913205488542161</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="8">
         <f t="shared" si="2"/>
         <v>2022.199140678425</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="8">
         <f t="shared" si="3"/>
         <v>22.19914067842501</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <f>'Price History'!A11</f>
         <v>45443</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="7">
         <f>'Price History'!B11</f>
         <v>104</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="9">
         <f t="shared" si="0"/>
         <v>4.8076923076923075</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="9">
         <f t="shared" si="4"/>
         <v>25.233946253939024</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="8">
         <f t="shared" si="5"/>
         <v>2500</v>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="7">
         <f t="shared" si="1"/>
         <v>99.072890733836346</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="8">
         <f t="shared" si="2"/>
         <v>2624.3304104096587</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="8">
         <f t="shared" si="3"/>
         <v>124.33041040965873</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <f>'Price History'!A12</f>
         <v>45473</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="7">
         <f>'Price History'!B12</f>
         <v>108</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="9">
         <f t="shared" si="0"/>
         <v>4.6296296296296298</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="9">
         <f t="shared" si="4"/>
         <v>29.863575883568654</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="8">
         <f t="shared" si="5"/>
         <v>3000</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="7">
         <f t="shared" si="1"/>
         <v>100.45682445050529</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="8">
         <f t="shared" si="2"/>
         <v>3225.2661954254145</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="8">
         <f t="shared" si="3"/>
         <v>225.26619542541448</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="6">
         <f>'Price History'!A13</f>
         <v>45504</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="7">
         <f>'Price History'!B13</f>
         <v>111</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="9">
         <f t="shared" si="0"/>
         <v>4.5045045045045047</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="9">
         <f t="shared" si="4"/>
         <v>34.36808038807316</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="8">
         <f t="shared" si="5"/>
         <v>3500</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="7">
         <f t="shared" si="1"/>
         <v>101.83868172092072</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="8">
         <f t="shared" si="2"/>
         <v>3814.8569230761209</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="8">
         <f t="shared" si="3"/>
         <v>314.85692307612089</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="6">
         <f>'Price History'!A14</f>
         <v>45535</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="7">
         <f>'Price History'!B14</f>
         <v>109</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="9">
         <f t="shared" si="0"/>
         <v>4.5871559633027523</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="9">
         <f t="shared" si="4"/>
         <v>38.955236351375916</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="8">
         <f t="shared" si="5"/>
         <v>4000</v>
       </c>
-      <c r="G9" s="9">
+      <c r="G9" s="7">
         <f t="shared" si="1"/>
         <v>102.68195946547552</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="8">
         <f t="shared" si="2"/>
         <v>4246.1207622999746</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="8">
         <f t="shared" si="3"/>
         <v>246.12076229997456</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="6">
         <f>'Price History'!A15</f>
         <v>45565</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="7">
         <f>'Price History'!B15</f>
         <v>105</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="9">
         <f t="shared" si="0"/>
         <v>4.7619047619047619</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="9">
         <f t="shared" si="4"/>
         <v>43.717141113280675</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="8">
         <f t="shared" si="5"/>
         <v>4500</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="7">
         <f t="shared" si="1"/>
         <v>102.93445283486209</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="8">
         <f t="shared" si="2"/>
         <v>4590.2998168944705</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="8">
         <f t="shared" si="3"/>
         <v>90.299816894470496</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="6">
         <f>'Price History'!A16</f>
         <v>45596</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="7">
         <f>'Price History'!B16</f>
         <v>101</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="9">
         <f t="shared" si="0"/>
         <v>4.9504950495049505</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="9">
         <f t="shared" si="4"/>
         <v>48.667636162785627</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="8">
         <f t="shared" si="5"/>
         <v>5000</v>
       </c>
-      <c r="G11" s="9">
+      <c r="G11" s="7">
         <f t="shared" si="1"/>
         <v>102.73767937435429</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="8">
         <f t="shared" si="2"/>
         <v>4915.4312524413481</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="8">
         <f t="shared" si="3"/>
         <v>-84.568747558651921</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
+      <c r="A12" s="6">
         <f>'Price History'!A17</f>
         <v>45626</v>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="7">
         <f>'Price History'!B17</f>
         <v>98</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="9">
         <f t="shared" si="0"/>
         <v>5.1020408163265305</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="9">
         <f t="shared" si="4"/>
         <v>53.769676979112155</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="8">
         <f t="shared" si="5"/>
         <v>5500</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="7">
         <f t="shared" si="1"/>
         <v>102.28813541387981</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="8">
         <f t="shared" si="2"/>
         <v>5269.4283439529909</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="8">
         <f t="shared" si="3"/>
         <v>-230.57165604700913</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <f>'Price History'!A18</f>
         <v>45657</v>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="7">
         <f>'Price History'!B18</f>
         <v>103</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="9">
         <f t="shared" si="0"/>
         <v>4.8543689320388346</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="9">
         <f t="shared" si="4"/>
         <v>58.624045911150986</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="8">
         <f t="shared" si="5"/>
         <v>6000</v>
       </c>
-      <c r="G13" s="9">
+      <c r="G13" s="7">
         <f t="shared" si="1"/>
         <v>102.34708141934519</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="8">
         <f t="shared" si="2"/>
         <v>6038.276728848552</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="8">
         <f t="shared" si="3"/>
         <v>38.276728848552011</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="6">
         <f>'Price History'!A19</f>
         <v>45688</v>
       </c>
-      <c r="B14" s="19">
+      <c r="B14" s="7">
         <f>'Price History'!B19</f>
         <v>107</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="9">
         <f t="shared" si="0"/>
         <v>4.6728971962616823</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="9">
         <f t="shared" si="4"/>
         <v>63.296943107412666</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="8">
         <f t="shared" si="5"/>
         <v>6500</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="7">
         <f t="shared" si="1"/>
         <v>102.69058316086024</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="8">
         <f t="shared" si="2"/>
         <v>6772.7729124931557</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="8">
         <f t="shared" si="3"/>
         <v>272.77291249315567</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="6">
         <f>'Price History'!A20</f>
         <v>45716</v>
       </c>
-      <c r="B15" s="19">
+      <c r="B15" s="7">
         <f>'Price History'!B20</f>
         <v>112</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="9">
         <f t="shared" si="0"/>
         <v>4.4642857142857144</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="9">
         <f t="shared" si="4"/>
         <v>67.761228821698381</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="8">
         <f t="shared" si="5"/>
         <v>7000</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G15" s="7">
         <f t="shared" si="1"/>
         <v>103.30391171652531</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="8">
         <f t="shared" si="2"/>
         <v>7589.2576280302183</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I15" s="8">
         <f t="shared" si="3"/>
         <v>589.25762803021826</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="6">
         <f>'Price History'!A21</f>
         <v>45747</v>
       </c>
-      <c r="B16" s="19">
+      <c r="B16" s="7">
         <f>'Price History'!B21</f>
         <v>116</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="9">
         <f t="shared" si="0"/>
         <v>4.3103448275862073</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="9">
         <f t="shared" si="4"/>
         <v>72.071573649284588</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="8">
         <f t="shared" si="5"/>
         <v>7500</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G16" s="7">
         <f t="shared" si="1"/>
         <v>104.06321966128525</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="8">
         <f t="shared" si="2"/>
         <v>8360.3025433170114</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I16" s="8">
         <f t="shared" si="3"/>
         <v>860.30254331701144</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="A17" s="6">
         <f>'Price History'!A22</f>
         <v>45777</v>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="7">
         <f>'Price History'!B22</f>
         <v>114</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="9">
         <f t="shared" si="0"/>
         <v>4.3859649122807021</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="9">
         <f t="shared" si="4"/>
         <v>76.457538561565286</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="8">
         <f t="shared" si="5"/>
         <v>8000</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="7">
         <f t="shared" si="1"/>
         <v>104.63324023383547</v>
       </c>
-      <c r="H17" s="10">
+      <c r="H17" s="8">
         <f t="shared" si="2"/>
         <v>8716.1593960184418</v>
       </c>
-      <c r="I17" s="10">
+      <c r="I17" s="8">
         <f t="shared" si="3"/>
         <v>716.15939601844184</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+      <c r="A18" s="6">
         <f>'Price History'!A23</f>
         <v>45808</v>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="7">
         <f>'Price History'!B23</f>
         <v>118</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="9">
         <f t="shared" si="0"/>
         <v>4.2372881355932206</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="9">
         <f t="shared" si="4"/>
         <v>80.694826697158504</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="8">
         <f t="shared" si="5"/>
         <v>8500</v>
       </c>
-      <c r="G18" s="9">
+      <c r="G18" s="7">
         <f t="shared" si="1"/>
         <v>105.33512925060052</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="8">
         <f t="shared" si="2"/>
         <v>9521.9895502647032</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I18" s="8">
         <f t="shared" si="3"/>
         <v>1021.9895502647032</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="6">
         <f>'Price History'!A24</f>
         <v>45838</v>
       </c>
-      <c r="B19" s="19">
+      <c r="B19" s="7">
         <f>'Price History'!B24</f>
         <v>121</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="9">
         <f t="shared" si="0"/>
         <v>4.1322314049586772</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="9">
         <f t="shared" si="4"/>
         <v>84.827058102117178</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="8">
         <f t="shared" si="5"/>
         <v>9000</v>
       </c>
-      <c r="G19" s="9">
+      <c r="G19" s="7">
         <f t="shared" si="1"/>
         <v>106.09822150339753</v>
       </c>
-      <c r="H19" s="10">
+      <c r="H19" s="8">
         <f t="shared" si="2"/>
         <v>10264.074030356178</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I19" s="8">
         <f t="shared" si="3"/>
         <v>1264.0740303561779</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="8">
+      <c r="A20" s="6">
         <f>'Price History'!A25</f>
         <v>45869</v>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="7">
         <f>'Price History'!B25</f>
         <v>125</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="9">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="9">
         <f t="shared" si="4"/>
         <v>88.827058102117178</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="8">
         <f t="shared" si="5"/>
         <v>9500</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="7">
         <f t="shared" si="1"/>
         <v>106.94939360795479</v>
       </c>
-      <c r="H20" s="10">
+      <c r="H20" s="8">
         <f t="shared" si="2"/>
         <v>11103.382262764648</v>
       </c>
-      <c r="I20" s="10">
+      <c r="I20" s="8">
         <f t="shared" si="3"/>
         <v>1603.3822627646477</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="A21" s="6">
         <f>'Price History'!A26</f>
         <v>45900</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="7">
         <f>'Price History'!B26</f>
         <v>123</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="9">
         <f t="shared" si="0"/>
         <v>4.0650406504065044</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="9">
         <f t="shared" si="4"/>
         <v>92.89209875252368</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="8">
         <f t="shared" si="5"/>
         <v>10000</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="7">
         <f t="shared" si="1"/>
         <v>107.65178238292653</v>
       </c>
-      <c r="H21" s="10">
+      <c r="H21" s="8">
         <f t="shared" si="2"/>
         <v>11425.728146560412</v>
       </c>
-      <c r="I21" s="10">
+      <c r="I21" s="8">
         <f t="shared" si="3"/>
         <v>1425.7281465604119</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="A22" s="6">
         <f>'Price History'!A27</f>
         <v>45930</v>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="7">
         <f>'Price History'!B27</f>
         <v>128</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="9">
         <f t="shared" si="0"/>
         <v>3.90625</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="9">
         <f t="shared" si="4"/>
         <v>96.79834875252368</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="8">
         <f t="shared" si="5"/>
         <v>10500</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="7">
         <f t="shared" si="1"/>
         <v>108.47292474838058</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="8">
         <f t="shared" si="2"/>
         <v>12390.188640323031</v>
       </c>
-      <c r="I22" s="10">
+      <c r="I22" s="8">
         <f t="shared" si="3"/>
         <v>1890.188640323031</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="A23" s="6">
         <f>'Price History'!A28</f>
         <v>45961</v>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="7">
         <f>'Price History'!B28</f>
         <v>131</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="9">
         <f t="shared" si="0"/>
         <v>3.8167938931297711</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="9">
         <f t="shared" si="4"/>
         <v>100.61514264565345</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="8">
         <f t="shared" si="5"/>
         <v>11000</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="7">
         <f t="shared" si="1"/>
         <v>109.32748004681379</v>
       </c>
-      <c r="H23" s="10">
+      <c r="H23" s="8">
         <f t="shared" si="2"/>
         <v>13180.583686580601</v>
       </c>
-      <c r="I23" s="10">
+      <c r="I23" s="8">
         <f t="shared" si="3"/>
         <v>2180.5836865806014</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
+      <c r="A24" s="6">
         <f>'Price History'!A29</f>
         <v>45991</v>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="7">
         <f>'Price History'!B29</f>
         <v>129</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="9">
         <f t="shared" si="0"/>
         <v>3.8759689922480618</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="9">
         <f t="shared" si="4"/>
         <v>104.49111163790151</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="8">
         <f t="shared" si="5"/>
         <v>11500</v>
       </c>
-      <c r="G24" s="9">
+      <c r="G24" s="7">
         <f t="shared" si="1"/>
         <v>110.05720792646507</v>
       </c>
-      <c r="H24" s="10">
+      <c r="H24" s="8">
         <f t="shared" si="2"/>
         <v>13479.353401289294</v>
       </c>
-      <c r="I24" s="10">
+      <c r="I24" s="8">
         <f t="shared" si="3"/>
         <v>1979.3534012892942</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="A25" s="6">
         <f>'Price History'!A30</f>
         <v>46022</v>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="7">
         <f>'Price History'!B30</f>
         <v>134</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <f>'Price History'!$B$1</f>
         <v>500</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="9">
         <f t="shared" si="0"/>
         <v>3.7313432835820897</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="9">
         <f t="shared" si="4"/>
         <v>108.2224549214836</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F25" s="8">
         <f t="shared" si="5"/>
         <v>12000</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="7">
         <f t="shared" si="1"/>
         <v>110.88271845899366</v>
       </c>
-      <c r="H25" s="10">
+      <c r="H25" s="8">
         <f t="shared" si="2"/>
         <v>14501.808959478803</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="8">
         <f t="shared" si="3"/>
         <v>2501.8089594788034</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="I2:I25">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{887E7235-FA1B-43C4-AC71-03F294ADCBE8}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{887E7235-FA1B-43C4-AC71-03F294ADCBE8}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF638EC6"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>I2:I25</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -5845,7 +4072,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -5856,7 +4083,7 @@
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="17" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -5873,625 +4100,625 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="6">
         <f>'Price History'!A7</f>
         <v>45322</v>
       </c>
-      <c r="B2" s="19">
+      <c r="B2" s="7">
         <f>'Price History'!B7</f>
         <v>102</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="9">
         <f t="shared" ref="D2:D25" si="0">$C$2/$B$2</f>
         <v>117.64705882352941</v>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="8">
         <f t="shared" ref="E2:E25" si="1">D2*B2</f>
         <v>12000</v>
       </c>
-      <c r="F2" s="10">
+      <c r="F2" s="8">
         <f t="shared" ref="F2:F25" si="2">E2-C2</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="6">
         <f>'Price History'!A8</f>
         <v>45351</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="7">
         <f>'Price History'!B8</f>
         <v>97</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="8">
         <f t="shared" si="1"/>
         <v>11411.764705882353</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="8">
         <f t="shared" si="2"/>
         <v>-588.23529411764684</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="6">
         <f>'Price History'!A9</f>
         <v>45382</v>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="7">
         <f>'Price History'!B9</f>
         <v>94</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="8">
         <f t="shared" si="1"/>
         <v>11058.823529411764</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="8">
         <f t="shared" si="2"/>
         <v>-941.17647058823604</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="6">
         <f>'Price History'!A10</f>
         <v>45412</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="7">
         <f>'Price History'!B10</f>
         <v>99</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="8">
         <f t="shared" si="1"/>
         <v>11647.058823529411</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="8">
         <f t="shared" si="2"/>
         <v>-352.9411764705892</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="6">
         <f>'Price History'!A11</f>
         <v>45443</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="7">
         <f>'Price History'!B11</f>
         <v>104</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="8">
         <f t="shared" si="1"/>
         <v>12235.294117647058</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="8">
         <f t="shared" si="2"/>
         <v>235.29411764705765</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="6">
         <f>'Price History'!A12</f>
         <v>45473</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="7">
         <f>'Price History'!B12</f>
         <v>108</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D7" s="11">
+      <c r="D7" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <f t="shared" si="1"/>
         <v>12705.882352941177</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="8">
         <f t="shared" si="2"/>
         <v>705.88235294117658</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="6">
         <f>'Price History'!A13</f>
         <v>45504</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="7">
         <f>'Price History'!B13</f>
         <v>111</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="8">
         <f t="shared" si="1"/>
         <v>13058.823529411764</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="8">
         <f t="shared" si="2"/>
         <v>1058.823529411764</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="6">
         <f>'Price History'!A14</f>
         <v>45535</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="7">
         <f>'Price History'!B14</f>
         <v>109</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D9" s="11">
+      <c r="D9" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="8">
         <f t="shared" si="1"/>
         <v>12823.529411764704</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="8">
         <f t="shared" si="2"/>
         <v>823.52941176470449</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="6">
         <f>'Price History'!A15</f>
         <v>45565</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="7">
         <f>'Price History'!B15</f>
         <v>105</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D10" s="11">
+      <c r="D10" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="8">
         <f t="shared" si="1"/>
         <v>12352.941176470587</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="8">
         <f t="shared" si="2"/>
         <v>352.94117647058738</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="6">
         <f>'Price History'!A16</f>
         <v>45596</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="7">
         <f>'Price History'!B16</f>
         <v>101</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="8">
         <f t="shared" si="1"/>
         <v>11882.35294117647</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="8">
         <f t="shared" si="2"/>
         <v>-117.64705882352973</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
+      <c r="A12" s="6">
         <f>'Price History'!A17</f>
         <v>45626</v>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="7">
         <f>'Price History'!B17</f>
         <v>98</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="8">
         <f t="shared" si="1"/>
         <v>11529.411764705881</v>
       </c>
-      <c r="F12" s="10">
+      <c r="F12" s="8">
         <f t="shared" si="2"/>
         <v>-470.58823529411893</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="6">
         <f>'Price History'!A18</f>
         <v>45657</v>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="7">
         <f>'Price History'!B18</f>
         <v>103</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="8">
         <f t="shared" si="1"/>
         <v>12117.647058823528</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="8">
         <f t="shared" si="2"/>
         <v>117.64705882352791</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="6">
         <f>'Price History'!A19</f>
         <v>45688</v>
       </c>
-      <c r="B14" s="19">
+      <c r="B14" s="7">
         <f>'Price History'!B19</f>
         <v>107</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="8">
         <f t="shared" si="1"/>
         <v>12588.235294117647</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="8">
         <f t="shared" si="2"/>
         <v>588.23529411764684</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="6">
         <f>'Price History'!A20</f>
         <v>45716</v>
       </c>
-      <c r="B15" s="19">
+      <c r="B15" s="7">
         <f>'Price History'!B20</f>
         <v>112</v>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="8">
         <f t="shared" si="1"/>
         <v>13176.470588235294</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="8">
         <f t="shared" si="2"/>
         <v>1176.4705882352937</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="6">
         <f>'Price History'!A21</f>
         <v>45747</v>
       </c>
-      <c r="B16" s="19">
+      <c r="B16" s="7">
         <f>'Price History'!B21</f>
         <v>116</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="8">
         <f t="shared" si="1"/>
         <v>13647.058823529411</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="8">
         <f t="shared" si="2"/>
         <v>1647.0588235294108</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="A17" s="6">
         <f>'Price History'!A22</f>
         <v>45777</v>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="7">
         <f>'Price History'!B22</f>
         <v>114</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="8">
         <f t="shared" si="1"/>
         <v>13411.764705882353</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="8">
         <f t="shared" si="2"/>
         <v>1411.7647058823532</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+      <c r="A18" s="6">
         <f>'Price History'!A23</f>
         <v>45808</v>
       </c>
-      <c r="B18" s="19">
+      <c r="B18" s="7">
         <f>'Price History'!B23</f>
         <v>118</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="8">
         <f t="shared" si="1"/>
         <v>13882.35294117647</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="8">
         <f t="shared" si="2"/>
         <v>1882.3529411764703</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="6">
         <f>'Price History'!A24</f>
         <v>45838</v>
       </c>
-      <c r="B19" s="19">
+      <c r="B19" s="7">
         <f>'Price History'!B24</f>
         <v>121</v>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="8">
         <f t="shared" si="1"/>
         <v>14235.294117647058</v>
       </c>
-      <c r="F19" s="10">
+      <c r="F19" s="8">
         <f t="shared" si="2"/>
         <v>2235.2941176470576</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="8">
+      <c r="A20" s="6">
         <f>'Price History'!A25</f>
         <v>45869</v>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="7">
         <f>'Price History'!B25</f>
         <v>125</v>
       </c>
-      <c r="C20" s="10">
+      <c r="C20" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="8">
         <f t="shared" si="1"/>
         <v>14705.882352941177</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="8">
         <f t="shared" si="2"/>
         <v>2705.8823529411766</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="A21" s="6">
         <f>'Price History'!A26</f>
         <v>45900</v>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="7">
         <f>'Price History'!B26</f>
         <v>123</v>
       </c>
-      <c r="C21" s="10">
+      <c r="C21" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E21" s="10">
+      <c r="E21" s="8">
         <f t="shared" si="1"/>
         <v>14470.588235294117</v>
       </c>
-      <c r="F21" s="10">
+      <c r="F21" s="8">
         <f t="shared" si="2"/>
         <v>2470.5882352941171</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="A22" s="6">
         <f>'Price History'!A27</f>
         <v>45930</v>
       </c>
-      <c r="B22" s="19">
+      <c r="B22" s="7">
         <f>'Price History'!B27</f>
         <v>128</v>
       </c>
-      <c r="C22" s="10">
+      <c r="C22" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E22" s="10">
+      <c r="E22" s="8">
         <f t="shared" si="1"/>
         <v>15058.823529411764</v>
       </c>
-      <c r="F22" s="10">
+      <c r="F22" s="8">
         <f t="shared" si="2"/>
         <v>3058.823529411764</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="A23" s="6">
         <f>'Price History'!A28</f>
         <v>45961</v>
       </c>
-      <c r="B23" s="19">
+      <c r="B23" s="7">
         <f>'Price History'!B28</f>
         <v>131</v>
       </c>
-      <c r="C23" s="10">
+      <c r="C23" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="8">
         <f t="shared" si="1"/>
         <v>15411.764705882351</v>
       </c>
-      <c r="F23" s="10">
+      <c r="F23" s="8">
         <f t="shared" si="2"/>
         <v>3411.7647058823513</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
+      <c r="A24" s="6">
         <f>'Price History'!A29</f>
         <v>45991</v>
       </c>
-      <c r="B24" s="19">
+      <c r="B24" s="7">
         <f>'Price History'!B29</f>
         <v>129</v>
       </c>
-      <c r="C24" s="10">
+      <c r="C24" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E24" s="10">
+      <c r="E24" s="8">
         <f t="shared" si="1"/>
         <v>15176.470588235294</v>
       </c>
-      <c r="F24" s="10">
+      <c r="F24" s="8">
         <f t="shared" si="2"/>
         <v>3176.4705882352937</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="A25" s="6">
         <f>'Price History'!A30</f>
         <v>46022</v>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="7">
         <f>'Price History'!B30</f>
         <v>134</v>
       </c>
-      <c r="C25" s="10">
+      <c r="C25" s="8">
         <f>'Price History'!$B$1*24</f>
         <v>12000</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="9">
         <f t="shared" si="0"/>
         <v>117.64705882352941</v>
       </c>
-      <c r="E25" s="10">
+      <c r="E25" s="8">
         <f t="shared" si="1"/>
         <v>15764.705882352941</v>
       </c>
-      <c r="F25" s="10">
+      <c r="F25" s="8">
         <f t="shared" si="2"/>
         <v>3764.7058823529405</v>
       </c>
@@ -6507,14 +4734,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="12">
+      <c r="B1" s="10">
         <f>'DCA Schedule'!F25</f>
         <v>12000</v>
       </c>
@@ -6523,7 +4750,7 @@
       <c r="A2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="10">
         <f>'DCA Schedule'!H25</f>
         <v>14501.808959478803</v>
       </c>
@@ -6532,7 +4759,7 @@
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="10">
         <f>'Lump Sum Comparison'!E25</f>
         <v>15764.705882352941</v>
       </c>
@@ -6541,7 +4768,7 @@
       <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="10">
         <f>'DCA Schedule'!I25</f>
         <v>2501.8089594788034</v>
       </c>
@@ -6550,7 +4777,7 @@
       <c r="A5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="10">
         <f>'Lump Sum Comparison'!F25</f>
         <v>3764.7058823529405</v>
       </c>
@@ -6559,7 +4786,7 @@
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="11">
         <f>'DCA Schedule'!G25</f>
         <v>110.88271845899366</v>
       </c>
@@ -6568,30 +4795,30 @@
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="11">
         <f>'Lump Sum Comparison'!B2</f>
         <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="14"/>
+      <c r="B8" s="1"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="14"/>
+      <c r="B9" s="1"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="1"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="12">
         <f>INDEX('Price History'!A7:A30,MATCH(MIN('Price History'!B7:B30),'Price History'!B7:B30,0))</f>
         <v>45382</v>
       </c>
@@ -6600,7 +4827,7 @@
       <c r="A12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="12">
         <f>INDEX('Price History'!A7:A30,MATCH(MIN('DCA Schedule'!I2:I25),'DCA Schedule'!I2:I25,0))</f>
         <v>45626</v>
       </c>
@@ -6609,7 +4836,7 @@
       <c r="A13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="16" t="str">
+      <c r="B13" s="13" t="str">
         <f>IF(B3&gt;B2,"Lump Sum","DCA")</f>
         <v>Lump Sum</v>
       </c>

</xml_diff>